<commit_message>
Reconnect the Section 1 answer workbooks
The workbooks existed on disk but nothing linked to them -- the links were lost
when the bank was trimmed and restored. Two workbooks also described questions
that no longer exist.

Adds the missing weighted-average builder, remaps the generator's numbering to
the questions as they now stand, drops five stale workbooks, and de-numbers the
titles so a renumbering does not invalidate them again.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q04.xlsx
+++ b/practice/answers/s1_q04.xlsx
@@ -17,10 +17,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MMM-YYYY"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,12 +54,6 @@
       <name val="Consolas"/>
       <color rgb="002F5D46"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0024302A"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -97,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,22 +101,27 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,26 +487,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q4 — Days between deliveries</t>
+          <t>Formatting changes the display, not the value</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Subtracting one date from another gives a number of days, because Excel stores dates as numbers. The result cell must be formatted as a NUMBER -- left as a date it shows a day in January 1900.</t>
+          <t>Column B holds the SAME number in every row -- 0.0842. Only the number format differs. Column D proves the stored value never changed.</t>
         </is>
       </c>
     </row>
@@ -515,137 +514,133 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Format applied</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Crop</t>
+          <t>Displayed as</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Days since previous</t>
+          <t>Number format</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>The formula in C</t>
+          <t>B x 1000</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>46279</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Canola</t>
-        </is>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.0842</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D5" s="8">
+        <f>B5*1000</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>46283</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Canola</t>
-        </is>
-      </c>
-      <c r="C6" s="8">
-        <f>A6-A5</f>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Number, 2 decimals</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="D6" s="8">
+        <f>B6*1000</f>
         <v/>
       </c>
-      <c r="D6" s="9">
-        <f>_xlfn.FORMULATEXT(C6)</f>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Percentage, 1 decimal</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D7" s="8">
+        <f>B7*1000</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>46288</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="C7" s="8">
-        <f>A7-A6</f>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>"$"#,##0.00</t>
+        </is>
+      </c>
+      <c r="D8" s="8">
+        <f>B8*1000</f>
         <v/>
       </c>
-      <c r="D7" s="9">
-        <f>_xlfn.FORMULATEXT(C7)</f>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Scientific</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>0.00E+00</t>
+        </is>
+      </c>
+      <c r="D9" s="8">
+        <f>B9*1000</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>46297</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="C8" s="8">
-        <f>A8-A7</f>
-        <v/>
-      </c>
-      <c r="D8" s="9">
-        <f>_xlfn.FORMULATEXT(C8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>46304</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Barley</t>
-        </is>
-      </c>
-      <c r="C9" s="8">
-        <f>A9-A8</f>
-        <v/>
-      </c>
-      <c r="D9" s="9">
-        <f>_xlfn.FORMULATEXT(C9)</f>
-        <v/>
-      </c>
-    </row>
     <row r="10" ht="18" customHeight="1"/>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>First to last</t>
-        </is>
-      </c>
-      <c r="C11" s="11">
-        <f>A9-A5</f>
-        <v/>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Every row in column D reads 84.20. The percentage row DISPLAYS 8.4% but still holds 0.0842 -- formatting never changes what a formula sees.</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1"/>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>25 days from the first delivery to the last. If a gap shows as a date like 04-Jan-1900, the cell is still formatted as a date -- change it to Number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>